<commit_message>
added new cracmm, edited mech info
</commit_message>
<xml_diff>
--- a/F0AM-4.3.0.1/Chem/mapping_mechs.xlsx
+++ b/F0AM-4.3.0.1/Chem/mapping_mechs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/USOS_shared/F0AM-4.3.0.1/Chem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F876A43C-59F9-E04D-A6B6-C1E9A59D780A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0B21ED-8522-B441-96A0-5EE7B9FA40C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6620" yWindow="1260" windowWidth="29220" windowHeight="20900" xr2:uid="{08BB61AC-5A18-114D-9375-14B9AF90892A}"/>
+    <workbookView xWindow="220" yWindow="700" windowWidth="38180" windowHeight="20900" xr2:uid="{08BB61AC-5A18-114D-9375-14B9AF90892A}"/>
   </bookViews>
   <sheets>
     <sheet name="CRACMM" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="240">
   <si>
     <t>CB6r5h</t>
   </si>
@@ -398,9 +398,6 @@
     <t>HC5</t>
   </si>
   <si>
-    <t>API</t>
-  </si>
-  <si>
     <t>Naphthalene</t>
   </si>
   <si>
@@ -461,9 +458,6 @@
     <t>Primary</t>
   </si>
   <si>
-    <t>Constrain</t>
-  </si>
-  <si>
     <t>N(=O)[O]</t>
   </si>
   <si>
@@ -650,9 +644,6 @@
     <t>styrene</t>
   </si>
   <si>
-    <t>prop-2-enal</t>
-  </si>
-  <si>
     <t>acrolein</t>
   </si>
   <si>
@@ -732,6 +723,39 @@
   </si>
   <si>
     <t>CRACMM lumped?</t>
+  </si>
+  <si>
+    <t>2-propenal</t>
+  </si>
+  <si>
+    <t>aromatic hydrocarbon</t>
+  </si>
+  <si>
+    <t>Constrain for CRACMM</t>
+  </si>
+  <si>
+    <t>API,LIM</t>
+  </si>
+  <si>
+    <t>CLNO2</t>
+  </si>
+  <si>
+    <t>aromatic aldehyde</t>
+  </si>
+  <si>
+    <t>benzaldehyde</t>
+  </si>
+  <si>
+    <t>InChI=1S/C7H6O/c8-6-7-4-2-1-3-5-7/h1-6H</t>
+  </si>
+  <si>
+    <t>C1=CC=C(C=C1)C=O</t>
+  </si>
+  <si>
+    <t>Acetonitrile_PTR</t>
+  </si>
+  <si>
+    <t>SLOWROC</t>
   </si>
 </sst>
 </file>
@@ -1105,7 +1129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D87BD187-C216-B54D-A8A1-FF7784763F8D}">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -1119,28 +1143,28 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C1" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
       </c>
       <c r="F1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I1" t="s">
         <v>2</v>
@@ -1149,18 +1173,18 @@
         <v>3</v>
       </c>
       <c r="K1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="L1" t="s">
-        <v>141</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D2" t="s">
         <v>92</v>
@@ -1181,15 +1205,15 @@
         <v>79</v>
       </c>
       <c r="K2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D3" t="s">
         <v>91</v>
@@ -1210,15 +1234,15 @@
         <v>81</v>
       </c>
       <c r="K3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>90</v>
@@ -1233,7 +1257,7 @@
         <v>119</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>10</v>
@@ -1242,15 +1266,18 @@
         <v>82</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>89</v>
@@ -1273,10 +1300,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>88</v>
@@ -1294,15 +1321,15 @@
         <v>36</v>
       </c>
       <c r="J6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>87</v>
@@ -1320,15 +1347,15 @@
         <v>37</v>
       </c>
       <c r="J7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>86</v>
@@ -1346,15 +1373,15 @@
         <v>42</v>
       </c>
       <c r="J8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B9" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>85</v>
@@ -1372,15 +1399,15 @@
         <v>44</v>
       </c>
       <c r="J9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>84</v>
@@ -1398,7 +1425,7 @@
         <v>46</v>
       </c>
       <c r="J10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -1412,10 +1439,10 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>93</v>
@@ -1433,12 +1460,12 @@
         <v>49</v>
       </c>
       <c r="J12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>94</v>
@@ -1450,18 +1477,18 @@
         <v>50</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>120</v>
+        <v>232</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B14" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>95</v>
@@ -1479,15 +1506,15 @@
         <v>52</v>
       </c>
       <c r="J14" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>96</v>
@@ -1505,15 +1532,15 @@
         <v>54</v>
       </c>
       <c r="J15" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B16" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>97</v>
@@ -1531,15 +1558,15 @@
         <v>55</v>
       </c>
       <c r="J16" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B17" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>102</v>
@@ -1560,12 +1587,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B18" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>98</v>
@@ -1583,15 +1610,15 @@
         <v>60</v>
       </c>
       <c r="J18" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B19" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>99</v>
@@ -1609,18 +1636,18 @@
         <v>62</v>
       </c>
       <c r="J19" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="K19" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B20" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>100</v>
@@ -1641,12 +1668,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B21" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>101</v>
@@ -1664,15 +1691,15 @@
         <v>66</v>
       </c>
       <c r="J21" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B22" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>104</v>
@@ -1683,19 +1710,22 @@
       <c r="F22" s="1" t="s">
         <v>67</v>
       </c>
+      <c r="G22" t="s">
+        <v>32</v>
+      </c>
       <c r="I22" t="s">
         <v>68</v>
       </c>
       <c r="J22" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B23" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>105</v>
@@ -1706,19 +1736,22 @@
       <c r="F23" s="1" t="s">
         <v>70</v>
       </c>
+      <c r="G23" t="s">
+        <v>33</v>
+      </c>
       <c r="I23" t="s">
         <v>69</v>
       </c>
       <c r="J23" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B24" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>103</v>
@@ -1729,16 +1762,19 @@
       <c r="F24" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="G24" t="s">
+        <v>233</v>
+      </c>
       <c r="I24" t="s">
         <v>72</v>
       </c>
       <c r="J24" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>106</v>
@@ -1749,16 +1785,19 @@
       <c r="F25" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="G25" t="s">
+        <v>31</v>
+      </c>
       <c r="I25" t="s">
         <v>74</v>
       </c>
       <c r="J25" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>107</v>
@@ -1769,215 +1808,277 @@
       <c r="F26" s="1" t="s">
         <v>75</v>
       </c>
+      <c r="G26" t="s">
+        <v>34</v>
+      </c>
       <c r="I26" t="s">
         <v>76</v>
       </c>
       <c r="J26" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>195</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>197</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>114</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>113</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.2">
+        <v>197</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>115</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G29" s="4" t="s">
         <v>116</v>
       </c>
       <c r="I29" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="J29" s="4" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="B30" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B30" t="s">
-        <v>204</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="F30" t="s">
-        <v>130</v>
-      </c>
-      <c r="G30" t="s">
-        <v>118</v>
-      </c>
-      <c r="I30" t="s">
+      <c r="B31" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="I31" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J31" s="2" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="K31" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="D31" t="s">
-        <v>122</v>
-      </c>
-      <c r="F31" t="s">
-        <v>121</v>
-      </c>
-      <c r="G31" t="s">
+      <c r="D32" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="I31" t="s">
+      <c r="F32" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J32" s="2" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
+      <c r="K32" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="J33" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="H32" s="2" t="s">
+      <c r="K33" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="M33" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="I32" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>220</v>
+      </c>
+      <c r="B34" t="s">
+        <v>221</v>
+      </c>
+      <c r="C34" t="s">
+        <v>219</v>
+      </c>
+      <c r="D34" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" t="s">
+        <v>132</v>
+      </c>
+      <c r="I34" t="s">
+        <v>223</v>
+      </c>
+      <c r="J34" t="s">
+        <v>222</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="M34" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>215</v>
+      </c>
+      <c r="B35" t="s">
+        <v>215</v>
+      </c>
+      <c r="D35" t="s">
+        <v>214</v>
+      </c>
+      <c r="G35" t="s">
+        <v>225</v>
+      </c>
+      <c r="H35" t="s">
+        <v>136</v>
+      </c>
+      <c r="I35" t="s">
         <v>216</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>223</v>
-      </c>
-      <c r="B34" t="s">
-        <v>224</v>
-      </c>
-      <c r="C34" t="s">
-        <v>222</v>
-      </c>
-      <c r="D34" t="s">
-        <v>132</v>
-      </c>
-      <c r="G34" t="s">
-        <v>133</v>
-      </c>
-      <c r="I34" t="s">
+      <c r="J35" t="s">
+        <v>217</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D36" t="s">
         <v>226</v>
       </c>
-      <c r="J34" t="s">
-        <v>225</v>
-      </c>
-      <c r="K34" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>218</v>
-      </c>
-      <c r="B35" t="s">
-        <v>218</v>
-      </c>
-      <c r="D35" t="s">
-        <v>217</v>
-      </c>
-      <c r="G35" t="s">
-        <v>228</v>
-      </c>
-      <c r="I35" t="s">
-        <v>219</v>
-      </c>
-      <c r="J35" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D36" t="s">
-        <v>229</v>
-      </c>
       <c r="G36" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H36" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="D37" t="s">
+        <v>238</v>
+      </c>
+      <c r="G37" t="s">
+        <v>239</v>
+      </c>
+      <c r="H37" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed photolysis rates for CRACMM, moved Cross section files from updated F0AM version
edited JBottomUp and cracmm3m_J_edited
</commit_message>
<xml_diff>
--- a/F0AM-4.3.0.1/Chem/mapping_mechs.xlsx
+++ b/F0AM-4.3.0.1/Chem/mapping_mechs.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/USOS_shared/F0AM-4.3.0.1/Chem/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u1545774\Documents\GitHub\USOS_shared\F0AM-4.3.0.1\Chem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0B21ED-8522-B441-96A0-5EE7B9FA40C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE059806-FF9E-45DB-A8BE-920372DE9296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="700" windowWidth="38180" windowHeight="20900" xr2:uid="{08BB61AC-5A18-114D-9375-14B9AF90892A}"/>
+    <workbookView xWindow="3720" yWindow="1260" windowWidth="19200" windowHeight="10092" xr2:uid="{08BB61AC-5A18-114D-9375-14B9AF90892A}"/>
   </bookViews>
   <sheets>
-    <sheet name="CRACMM" sheetId="2" r:id="rId1"/>
+    <sheet name="F0AM_InitConc" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,16 +27,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="263">
   <si>
     <t>CB6r5h</t>
   </si>
@@ -95,9 +96,6 @@
     <t>PANX</t>
   </si>
   <si>
-    <t>NOx</t>
-  </si>
-  <si>
     <t>ISOP</t>
   </si>
   <si>
@@ -179,9 +177,6 @@
     <t>InChI=1S/C3H5NO5/c1-2-3(5)8-9-4(6)7/h2H2,1H3</t>
   </si>
   <si>
-    <t>NOx Family</t>
-  </si>
-  <si>
     <t>Isoprene</t>
   </si>
   <si>
@@ -587,9 +582,6 @@
     <t>chlorine</t>
   </si>
   <si>
-    <t>chlorine nitrite</t>
-  </si>
-  <si>
     <t>bromine chloride, bromine monochloride, bromochloride</t>
   </si>
   <si>
@@ -731,9 +723,6 @@
     <t>aromatic hydrocarbon</t>
   </si>
   <si>
-    <t>Constrain for CRACMM</t>
-  </si>
-  <si>
     <t>API,LIM</t>
   </si>
   <si>
@@ -756,13 +745,94 @@
   </si>
   <si>
     <t>SLOWROC</t>
+  </si>
+  <si>
+    <t>CRACMM Notes</t>
+  </si>
+  <si>
+    <t>GEOS-Chem</t>
+  </si>
+  <si>
+    <t>HNO2</t>
+  </si>
+  <si>
+    <t>MTPA</t>
+  </si>
+  <si>
+    <t>GEOS-Chem Notes</t>
+  </si>
+  <si>
+    <t>MTPO?</t>
+  </si>
+  <si>
+    <t>TOLU</t>
+  </si>
+  <si>
+    <t>CH2O</t>
+  </si>
+  <si>
+    <t>HCOOH</t>
+  </si>
+  <si>
+    <t>Br2</t>
+  </si>
+  <si>
+    <t>Cl2</t>
+  </si>
+  <si>
+    <t>nitryl chloride, chlorine nitrite</t>
+  </si>
+  <si>
+    <t>ClNO2</t>
+  </si>
+  <si>
+    <t>BrCl</t>
+  </si>
+  <si>
+    <t>BrO</t>
+  </si>
+  <si>
+    <t>GEOS-Chem Explicit?</t>
+  </si>
+  <si>
+    <t>InChI=1S/C10H16/c1-7-4-5-8-6-9(7)10(8,2)3/h4,8-9H,5-6H2,1-3H3;InChI=1S/C10H16/c1-7-4-5-8-6-9(7)10(8,2)3/h8-9H,1,4-6H2,2-3H3;InChI=1S/C10H16/c1-7(2)10-5-4-8(3)9(10)6-10/h7,9H,3-6H2,1-2H3;InChI=1S/C10H16/c1-7-4-5-8-9(6-7)10(8,2)3/h4,8-9H,5-6H2,1-3H3</t>
+  </si>
+  <si>
+    <t>STYR</t>
+  </si>
+  <si>
+    <t>ACR</t>
+  </si>
+  <si>
+    <t>NAP</t>
+  </si>
+  <si>
+    <t>MVK,MACR</t>
+  </si>
+  <si>
+    <t>InChI=1S/C2H3N/c1-2-3/h1H3</t>
+  </si>
+  <si>
+    <t>CC#N</t>
+  </si>
+  <si>
+    <t>Paper for Primary</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> https://doi.org/10.1029/JD091iD03p04003</t>
+  </si>
+  <si>
+    <t>acetonitrile</t>
+  </si>
+  <si>
+    <t>https://www.atsdr.cdc.gov/toxprofiles/tp67-c1.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -774,6 +844,14 @@
       <sz val="12"/>
       <name val="Consolas"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -805,18 +883,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1129,65 +1212,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D87BD187-C216-B54D-A8A1-FF7784763F8D}">
-  <dimension ref="A1:M37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:S36"/>
+  <sheetFormatPr defaultColWidth="10.69921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="30.6640625" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="47.33203125" hidden="1" customWidth="1"/>
-    <col min="7" max="8" width="18.6640625" customWidth="1"/>
+    <col min="2" max="3" width="22.796875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="19.8984375" customWidth="1"/>
+    <col min="5" max="5" width="10.796875" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="47.296875" hidden="1" customWidth="1"/>
+    <col min="7" max="9" width="18.69921875" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="18.69921875" customWidth="1"/>
+    <col min="11" max="12" width="18.69921875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="18.69921875" customWidth="1"/>
+    <col min="14" max="15" width="10.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C1" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
       </c>
       <c r="F1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G1" t="s">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="I1" t="s">
+        <v>225</v>
+      </c>
+      <c r="J1" t="s">
+        <v>237</v>
+      </c>
+      <c r="K1" t="s">
+        <v>240</v>
+      </c>
+      <c r="L1" t="s">
+        <v>251</v>
+      </c>
+      <c r="N1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" t="s">
+      <c r="O1" t="s">
         <v>3</v>
       </c>
-      <c r="K1" t="s">
-        <v>139</v>
-      </c>
-      <c r="L1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="P1" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
         <v>5</v>
@@ -1198,25 +1296,31 @@
       <c r="G2" t="s">
         <v>5</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" t="s">
         <v>4</v>
       </c>
-      <c r="J2" t="s">
-        <v>79</v>
-      </c>
-      <c r="K2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O2" t="s">
+        <v>77</v>
+      </c>
+      <c r="P2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E3" t="s">
         <v>11</v>
@@ -1227,271 +1331,358 @@
       <c r="G3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" t="s">
         <v>12</v>
       </c>
-      <c r="J3" t="s">
-        <v>81</v>
-      </c>
-      <c r="K3" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="O3" t="s">
+        <v>79</v>
+      </c>
+      <c r="P3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="G4" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4"/>
+      <c r="N4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O4" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E5" t="s">
         <v>13</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
       </c>
-      <c r="I5" t="s">
-        <v>35</v>
-      </c>
       <c r="J5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
         <v>14</v>
       </c>
-      <c r="I6" t="s">
-        <v>36</v>
-      </c>
       <c r="J6" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" t="s">
+        <v>35</v>
+      </c>
+      <c r="O6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E7" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
       </c>
-      <c r="I7" t="s">
-        <v>37</v>
-      </c>
       <c r="J7" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>238</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" t="s">
+        <v>36</v>
+      </c>
+      <c r="O7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G8" t="s">
         <v>16</v>
       </c>
-      <c r="I8" t="s">
-        <v>42</v>
-      </c>
       <c r="J8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="N8" t="s">
+        <v>41</v>
+      </c>
+      <c r="O8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E9" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
       </c>
-      <c r="I9" t="s">
-        <v>44</v>
-      </c>
       <c r="J9" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="N9" t="s">
+        <v>43</v>
+      </c>
+      <c r="O9" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E10" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" t="s">
+        <v>81</v>
+      </c>
+      <c r="J10" t="s">
+        <v>81</v>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" t="s">
         <v>45</v>
       </c>
-      <c r="G10" t="s">
-        <v>83</v>
-      </c>
-      <c r="I10" t="s">
-        <v>46</v>
-      </c>
-      <c r="J10" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="D11" s="1"/>
+      <c r="O10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>221</v>
+      </c>
+      <c r="B11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>91</v>
+      </c>
       <c r="E11" t="s">
         <v>19</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" t="s">
+        <v>19</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>224</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="O11" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="L12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N12" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>157</v>
+      </c>
+      <c r="B13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" t="s">
+        <v>21</v>
+      </c>
+      <c r="J13" t="s">
+        <v>21</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="N13" t="s">
+        <v>50</v>
+      </c>
+      <c r="O13" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>158</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="E12" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" t="s">
-        <v>49</v>
-      </c>
-      <c r="J12" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="B14" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>159</v>
-      </c>
-      <c r="B14" t="s">
-        <v>159</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="E14" t="s">
         <v>22</v>
@@ -1500,76 +1691,94 @@
         <v>51</v>
       </c>
       <c r="G14" t="s">
+        <v>106</v>
+      </c>
+      <c r="J14" t="s">
         <v>22</v>
       </c>
-      <c r="I14" t="s">
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="N14" t="s">
         <v>52</v>
       </c>
-      <c r="J14" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O14" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E15" t="s">
         <v>23</v>
       </c>
       <c r="F15" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" t="s">
+        <v>242</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="N15" t="s">
         <v>53</v>
       </c>
-      <c r="G15" t="s">
-        <v>108</v>
-      </c>
-      <c r="I15" t="s">
-        <v>54</v>
-      </c>
-      <c r="J15" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E16" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" t="s">
+        <v>107</v>
+      </c>
+      <c r="J16" t="s">
+        <v>107</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="N16" t="s">
         <v>56</v>
       </c>
-      <c r="G16" t="s">
-        <v>24</v>
-      </c>
-      <c r="I16" t="s">
-        <v>55</v>
-      </c>
-      <c r="J16" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="B17" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E17" t="s">
         <v>25</v>
@@ -1578,24 +1787,30 @@
         <v>57</v>
       </c>
       <c r="G17" t="s">
-        <v>109</v>
-      </c>
-      <c r="I17" t="s">
+        <v>108</v>
+      </c>
+      <c r="J17" t="s">
+        <v>25</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="N17" t="s">
         <v>58</v>
       </c>
-      <c r="J17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O17" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B18" t="s">
         <v>167</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E18" t="s">
         <v>26</v>
@@ -1604,24 +1819,33 @@
         <v>59</v>
       </c>
       <c r="G18" t="s">
-        <v>110</v>
-      </c>
-      <c r="I18" t="s">
+        <v>109</v>
+      </c>
+      <c r="J18" t="s">
+        <v>109</v>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="N18" t="s">
         <v>60</v>
       </c>
-      <c r="J18" t="s">
+      <c r="O18" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="P18" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>187</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
         <v>169</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E19" t="s">
         <v>27</v>
@@ -1630,27 +1854,30 @@
         <v>61</v>
       </c>
       <c r="G19" t="s">
-        <v>111</v>
-      </c>
-      <c r="I19" t="s">
+        <v>75</v>
+      </c>
+      <c r="J19" t="s">
+        <v>243</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="N19" t="s">
         <v>62</v>
       </c>
-      <c r="J19" t="s">
+      <c r="O19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>170</v>
       </c>
-      <c r="K19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>171</v>
-      </c>
       <c r="B20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E20" t="s">
         <v>28</v>
@@ -1659,102 +1886,123 @@
         <v>63</v>
       </c>
       <c r="G20" t="s">
-        <v>77</v>
-      </c>
-      <c r="I20" t="s">
+        <v>110</v>
+      </c>
+      <c r="J20" t="s">
+        <v>244</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="N20" t="s">
         <v>64</v>
       </c>
-      <c r="J20" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O20" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="B21" t="s">
         <v>172</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>65</v>
       </c>
       <c r="G21" t="s">
-        <v>112</v>
-      </c>
-      <c r="I21" t="s">
+        <v>31</v>
+      </c>
+      <c r="J21" t="s">
+        <v>245</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="N21" t="s">
         <v>66</v>
       </c>
-      <c r="J21" t="s">
+      <c r="O21" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B22" t="s">
         <v>174</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E22" t="s">
         <v>32</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G22" t="s">
         <v>32</v>
       </c>
-      <c r="I22" t="s">
-        <v>68</v>
-      </c>
       <c r="J22" t="s">
+        <v>246</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="N22" t="s">
+        <v>67</v>
+      </c>
+      <c r="O22" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>182</v>
+        <v>247</v>
       </c>
       <c r="B23" t="s">
         <v>176</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E23" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F23" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G23" t="s">
+        <v>229</v>
+      </c>
+      <c r="J23" t="s">
+        <v>248</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="N23" t="s">
         <v>70</v>
       </c>
-      <c r="G23" t="s">
-        <v>33</v>
-      </c>
-      <c r="I23" t="s">
-        <v>69</v>
-      </c>
-      <c r="J23" t="s">
+      <c r="O23" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>183</v>
-      </c>
-      <c r="B24" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E24" t="s">
         <v>30</v>
@@ -1763,140 +2011,185 @@
         <v>71</v>
       </c>
       <c r="G24" t="s">
-        <v>233</v>
-      </c>
-      <c r="I24" t="s">
+        <v>30</v>
+      </c>
+      <c r="J24" t="s">
+        <v>249</v>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+      <c r="N24" t="s">
         <v>72</v>
       </c>
-      <c r="J24" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="O24" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E25" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>73</v>
       </c>
       <c r="G25" t="s">
-        <v>31</v>
-      </c>
-      <c r="I25" t="s">
+        <v>33</v>
+      </c>
+      <c r="J25" t="s">
+        <v>250</v>
+      </c>
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
+      <c r="N25" t="s">
         <v>74</v>
       </c>
-      <c r="J25" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="O25" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="L27" t="b">
+        <v>1</v>
+      </c>
+      <c r="M27"/>
+      <c r="N27" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="O27" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E26" t="s">
-        <v>34</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G26" t="s">
-        <v>34</v>
-      </c>
-      <c r="I26" t="s">
-        <v>76</v>
-      </c>
-      <c r="J26" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="P27" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="L28" t="b">
+        <v>1</v>
+      </c>
+      <c r="M28"/>
+      <c r="N28" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="O28" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="J28" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="K28" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
+      <c r="P28" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="L29" t="b">
+        <v>1</v>
+      </c>
+      <c r="M29"/>
+      <c r="N29" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="I29" s="4" t="s">
+      <c r="O29" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="J29" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="K29" s="4" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="P29" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>202</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>117</v>
+        <v>202</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>119</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I30" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="N30" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="O30" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="P30" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q30" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="S30" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>205</v>
       </c>
@@ -1907,181 +2200,182 @@
         <v>121</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>122</v>
       </c>
       <c r="I31" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="O31" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="K31" s="2" t="s">
+      <c r="P31" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="S31" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="M31" s="2" t="s">
+    </row>
+    <row r="32" spans="1:19" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="O32" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="P32" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="S32" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>217</v>
+      </c>
+      <c r="B33" t="s">
+        <v>218</v>
+      </c>
+      <c r="C33" t="s">
+        <v>216</v>
+      </c>
+      <c r="D33" t="s">
+        <v>129</v>
+      </c>
+      <c r="G33" t="s">
+        <v>130</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="N33" t="s">
+        <v>220</v>
+      </c>
+      <c r="O33" t="s">
+        <v>219</v>
+      </c>
+      <c r="P33" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q33" s="2"/>
+      <c r="S33" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>212</v>
+      </c>
+      <c r="B34" t="s">
+        <v>212</v>
+      </c>
+      <c r="D34" t="s">
+        <v>211</v>
+      </c>
+      <c r="G34" t="s">
+        <v>222</v>
+      </c>
+      <c r="I34" t="s">
+        <v>134</v>
+      </c>
+      <c r="N34" t="s">
+        <v>213</v>
+      </c>
+      <c r="O34" t="s">
+        <v>214</v>
+      </c>
+      <c r="P34" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q34" s="2"/>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D35" t="s">
+        <v>223</v>
+      </c>
+      <c r="G35" t="s">
+        <v>224</v>
+      </c>
+      <c r="I35" t="s">
+        <v>134</v>
+      </c>
+      <c r="J35" t="s">
+        <v>224</v>
+      </c>
+      <c r="L35" t="b">
+        <v>1</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="O35" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="P35" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q35" s="2"/>
+      <c r="S35" s="2" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="32" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>220</v>
-      </c>
-      <c r="B34" t="s">
-        <v>221</v>
-      </c>
-      <c r="C34" t="s">
-        <v>219</v>
-      </c>
-      <c r="D34" t="s">
-        <v>131</v>
-      </c>
-      <c r="G34" t="s">
-        <v>132</v>
-      </c>
-      <c r="I34" t="s">
-        <v>223</v>
-      </c>
-      <c r="J34" t="s">
-        <v>222</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="M34" t="s">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D36" t="s">
+        <v>234</v>
+      </c>
+      <c r="G36" t="s">
+        <v>235</v>
+      </c>
+      <c r="I36" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>215</v>
-      </c>
-      <c r="B35" t="s">
-        <v>215</v>
-      </c>
-      <c r="D35" t="s">
-        <v>214</v>
-      </c>
-      <c r="G35" t="s">
-        <v>225</v>
-      </c>
-      <c r="H35" t="s">
-        <v>136</v>
-      </c>
-      <c r="I35" t="s">
-        <v>216</v>
-      </c>
-      <c r="J35" t="s">
-        <v>217</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A36" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="D36" t="s">
-        <v>226</v>
-      </c>
-      <c r="G36" t="s">
-        <v>227</v>
-      </c>
-      <c r="H36" t="s">
-        <v>136</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D37" t="s">
-        <v>238</v>
-      </c>
-      <c r="G37" t="s">
-        <v>239</v>
-      </c>
-      <c r="H37" t="s">
-        <v>136</v>
+      <c r="N36" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="O36" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="P36" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>260</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="Q30" r:id="rId1" xr:uid="{84EF3E6B-2376-462F-A4BA-FAA0E914BC7F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
edited mapping mechs file
</commit_message>
<xml_diff>
--- a/F0AM-4.3.0.1/Chem/mapping_mechs.xlsx
+++ b/F0AM-4.3.0.1/Chem/mapping_mechs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanessasun/Documents/phd/utah/research/USOS_shared/F0AM-4.3.0.1/Chem/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA0B21ED-8522-B441-96A0-5EE7B9FA40C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9B3061-03B6-1741-A91E-42354516E497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="700" windowWidth="38180" windowHeight="20900" xr2:uid="{08BB61AC-5A18-114D-9375-14B9AF90892A}"/>
+    <workbookView minimized="1" xWindow="220" yWindow="700" windowWidth="38180" windowHeight="20900" xr2:uid="{08BB61AC-5A18-114D-9375-14B9AF90892A}"/>
   </bookViews>
   <sheets>
     <sheet name="CRACMM" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="245">
   <si>
     <t>CB6r5h</t>
   </si>
@@ -756,6 +756,21 @@
   </si>
   <si>
     <t>SLOWROC</t>
+  </si>
+  <si>
+    <t>acetonitrile</t>
+  </si>
+  <si>
+    <t>CC#N</t>
+  </si>
+  <si>
+    <t>InChI=1S/C2H3N/c1-2-3/h1H3</t>
+  </si>
+  <si>
+    <t>acetonitrile,methyl cyanide</t>
+  </si>
+  <si>
+    <t>ISO</t>
   </si>
 </sst>
 </file>
@@ -1454,7 +1469,7 @@
         <v>48</v>
       </c>
       <c r="G12" t="s">
-        <v>20</v>
+        <v>244</v>
       </c>
       <c r="I12" t="s">
         <v>49</v>
@@ -2071,6 +2086,12 @@
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>240</v>
+      </c>
       <c r="D37" t="s">
         <v>238</v>
       </c>
@@ -2079,6 +2100,12 @@
       </c>
       <c r="H37" t="s">
         <v>136</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>